<commit_message>
Fix: set all option C scores to 3 across GRI 1/2/3
84 questions had C=4; corrected to C=3 so every question
follows the A=6 B=4 C=3 D=0 scoring pattern.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sustindex-/data/GRI_Questionnaire_v4_STRUCTURED.xlsx
+++ b/sustindex-/data/GRI_Questionnaire_v4_STRUCTURED.xlsx
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="I8" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J8" s="2" t="n"/>
       <c r="K8" s="2" t="n"/>
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="I12" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J12" s="2" t="n"/>
       <c r="K12" s="2" t="n"/>
@@ -1197,7 +1197,7 @@
         </is>
       </c>
       <c r="I25" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J25" s="2" t="n"/>
       <c r="K25" s="2" t="n"/>
@@ -1311,7 +1311,7 @@
         </is>
       </c>
       <c r="I29" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J29" s="2" t="n"/>
       <c r="K29" s="2" t="n"/>
@@ -1669,7 +1669,7 @@
         </is>
       </c>
       <c r="I42" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J42" s="2" t="n"/>
       <c r="K42" s="2" t="n"/>
@@ -1783,7 +1783,7 @@
         </is>
       </c>
       <c r="I46" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J46" s="2" t="n"/>
       <c r="K46" s="2" t="n"/>
@@ -2027,7 +2027,7 @@
         </is>
       </c>
       <c r="I55" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J55" s="2" t="n"/>
       <c r="K55" s="2" t="n"/>
@@ -2141,7 +2141,7 @@
         </is>
       </c>
       <c r="I59" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J59" s="2" t="n"/>
       <c r="K59" s="2" t="n"/>
@@ -2255,7 +2255,7 @@
         </is>
       </c>
       <c r="I63" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J63" s="2" t="n"/>
       <c r="K63" s="2" t="n"/>
@@ -2369,7 +2369,7 @@
         </is>
       </c>
       <c r="I67" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J67" s="2" t="n"/>
       <c r="K67" s="2" t="n"/>
@@ -2613,7 +2613,7 @@
         </is>
       </c>
       <c r="I76" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J76" s="2" t="n"/>
       <c r="K76" s="2" t="n"/>
@@ -2727,7 +2727,7 @@
         </is>
       </c>
       <c r="I80" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J80" s="2" t="n"/>
       <c r="K80" s="2" t="n"/>
@@ -3085,7 +3085,7 @@
         </is>
       </c>
       <c r="I93" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J93" s="2" t="n"/>
       <c r="K93" s="2" t="n"/>
@@ -3199,7 +3199,7 @@
         </is>
       </c>
       <c r="I97" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J97" s="2" t="n"/>
       <c r="K97" s="2" t="n"/>
@@ -4029,7 +4029,7 @@
         </is>
       </c>
       <c r="I127" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J127" s="2" t="n"/>
       <c r="K127" s="2" t="n"/>
@@ -4143,7 +4143,7 @@
         </is>
       </c>
       <c r="I131" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J131" s="2" t="n"/>
       <c r="K131" s="2" t="n"/>
@@ -5829,7 +5829,7 @@
         </is>
       </c>
       <c r="I8" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J8" s="2" t="n"/>
       <c r="K8" s="2" t="n"/>
@@ -5943,7 +5943,7 @@
         </is>
       </c>
       <c r="I12" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J12" s="2" t="n"/>
       <c r="K12" s="2" t="n"/>
@@ -6187,7 +6187,7 @@
         </is>
       </c>
       <c r="I21" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J21" s="2" t="n"/>
       <c r="K21" s="2" t="n"/>
@@ -6301,7 +6301,7 @@
         </is>
       </c>
       <c r="I25" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J25" s="2" t="n"/>
       <c r="K25" s="2" t="n"/>
@@ -6415,7 +6415,7 @@
         </is>
       </c>
       <c r="I29" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J29" s="2" t="n"/>
       <c r="K29" s="2" t="n"/>
@@ -6529,7 +6529,7 @@
         </is>
       </c>
       <c r="I33" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J33" s="2" t="n"/>
       <c r="K33" s="2" t="n"/>
@@ -6773,7 +6773,7 @@
         </is>
       </c>
       <c r="I42" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J42" s="2" t="n"/>
       <c r="K42" s="2" t="n"/>
@@ -6887,7 +6887,7 @@
         </is>
       </c>
       <c r="I46" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J46" s="2" t="n"/>
       <c r="K46" s="2" t="n"/>
@@ -7245,7 +7245,7 @@
         </is>
       </c>
       <c r="I59" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J59" s="2" t="n"/>
       <c r="K59" s="2" t="n"/>
@@ -7359,7 +7359,7 @@
         </is>
       </c>
       <c r="I63" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J63" s="2" t="n"/>
       <c r="K63" s="2" t="n"/>
@@ -7717,7 +7717,7 @@
         </is>
       </c>
       <c r="I76" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J76" s="2" t="n"/>
       <c r="K76" s="2" t="n"/>
@@ -7831,7 +7831,7 @@
         </is>
       </c>
       <c r="I80" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J80" s="2" t="n"/>
       <c r="K80" s="2" t="n"/>
@@ -8679,7 +8679,7 @@
         </is>
       </c>
       <c r="I111" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J111" s="2" t="n"/>
       <c r="K111" s="2" t="n"/>
@@ -8793,7 +8793,7 @@
         </is>
       </c>
       <c r="I115" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J115" s="2" t="n"/>
       <c r="K115" s="2" t="n"/>
@@ -9151,7 +9151,7 @@
         </is>
       </c>
       <c r="I128" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J128" s="2" t="n"/>
       <c r="K128" s="2" t="n"/>
@@ -9265,7 +9265,7 @@
         </is>
       </c>
       <c r="I132" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J132" s="2" t="n"/>
       <c r="K132" s="2" t="n"/>
@@ -9623,7 +9623,7 @@
         </is>
       </c>
       <c r="I145" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J145" s="2" t="n"/>
       <c r="K145" s="2" t="n"/>
@@ -9737,7 +9737,7 @@
         </is>
       </c>
       <c r="I149" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J149" s="2" t="n"/>
       <c r="K149" s="2" t="n"/>
@@ -10095,7 +10095,7 @@
         </is>
       </c>
       <c r="I162" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J162" s="2" t="n"/>
       <c r="K162" s="2" t="n"/>
@@ -10209,7 +10209,7 @@
         </is>
       </c>
       <c r="I166" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J166" s="2" t="n"/>
       <c r="K166" s="2" t="n"/>
@@ -11039,7 +11039,7 @@
         </is>
       </c>
       <c r="I196" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J196" s="2" t="n"/>
       <c r="K196" s="2" t="n"/>
@@ -11153,7 +11153,7 @@
         </is>
       </c>
       <c r="I200" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J200" s="2" t="n"/>
       <c r="K200" s="2" t="n"/>
@@ -11511,7 +11511,7 @@
         </is>
       </c>
       <c r="I213" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J213" s="2" t="n"/>
       <c r="K213" s="2" t="n"/>
@@ -11625,7 +11625,7 @@
         </is>
       </c>
       <c r="I217" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J217" s="2" t="n"/>
       <c r="K217" s="2" t="n"/>
@@ -11983,7 +11983,7 @@
         </is>
       </c>
       <c r="I230" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J230" s="2" t="n"/>
       <c r="K230" s="2" t="n"/>
@@ -12097,7 +12097,7 @@
         </is>
       </c>
       <c r="I234" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J234" s="2" t="n"/>
       <c r="K234" s="2" t="n"/>
@@ -12455,7 +12455,7 @@
         </is>
       </c>
       <c r="I247" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J247" s="2" t="n"/>
       <c r="K247" s="2" t="n"/>
@@ -12569,7 +12569,7 @@
         </is>
       </c>
       <c r="I251" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J251" s="2" t="n"/>
       <c r="K251" s="2" t="n"/>
@@ -15281,7 +15281,7 @@
         </is>
       </c>
       <c r="I4" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J4" s="2" t="n"/>
       <c r="K4" s="2" t="n"/>
@@ -15395,7 +15395,7 @@
         </is>
       </c>
       <c r="I8" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J8" s="2" t="n"/>
       <c r="K8" s="2" t="n"/>
@@ -15509,7 +15509,7 @@
         </is>
       </c>
       <c r="I12" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J12" s="2" t="n"/>
       <c r="K12" s="2" t="n"/>
@@ -15623,7 +15623,7 @@
         </is>
       </c>
       <c r="I16" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J16" s="2" t="n"/>
       <c r="K16" s="2" t="n"/>
@@ -15867,7 +15867,7 @@
         </is>
       </c>
       <c r="I25" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J25" s="2" t="n"/>
       <c r="K25" s="2" t="n"/>
@@ -15981,7 +15981,7 @@
         </is>
       </c>
       <c r="I29" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J29" s="2" t="n"/>
       <c r="K29" s="2" t="n"/>
@@ -16225,7 +16225,7 @@
         </is>
       </c>
       <c r="I38" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J38" s="2" t="n"/>
       <c r="K38" s="2" t="n"/>
@@ -16339,7 +16339,7 @@
         </is>
       </c>
       <c r="I42" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J42" s="2" t="n"/>
       <c r="K42" s="2" t="n"/>
@@ -16453,7 +16453,7 @@
         </is>
       </c>
       <c r="I46" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J46" s="2" t="n"/>
       <c r="K46" s="2" t="n"/>
@@ -16567,7 +16567,7 @@
         </is>
       </c>
       <c r="I50" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J50" s="2" t="n"/>
       <c r="K50" s="2" t="n"/>
@@ -17169,7 +17169,7 @@
         </is>
       </c>
       <c r="I72" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J72" s="2" t="n"/>
       <c r="K72" s="2" t="n"/>
@@ -17283,7 +17283,7 @@
         </is>
       </c>
       <c r="I76" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J76" s="2" t="n"/>
       <c r="K76" s="2" t="n"/>
@@ -17397,7 +17397,7 @@
         </is>
       </c>
       <c r="I80" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J80" s="2" t="n"/>
       <c r="K80" s="2" t="n"/>
@@ -17511,7 +17511,7 @@
         </is>
       </c>
       <c r="I84" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J84" s="2" t="n"/>
       <c r="K84" s="2" t="n"/>
@@ -17755,7 +17755,7 @@
         </is>
       </c>
       <c r="I93" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J93" s="2" t="n"/>
       <c r="K93" s="2" t="n"/>
@@ -17869,7 +17869,7 @@
         </is>
       </c>
       <c r="I97" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J97" s="2" t="n"/>
       <c r="K97" s="2" t="n"/>
@@ -18227,7 +18227,7 @@
         </is>
       </c>
       <c r="I110" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J110" s="2" t="n"/>
       <c r="K110" s="2" t="n"/>
@@ -18341,7 +18341,7 @@
         </is>
       </c>
       <c r="I114" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J114" s="2" t="n"/>
       <c r="K114" s="2" t="n"/>
@@ -18699,7 +18699,7 @@
         </is>
       </c>
       <c r="I127" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J127" s="2" t="n"/>
       <c r="K127" s="2" t="n"/>
@@ -18813,7 +18813,7 @@
         </is>
       </c>
       <c r="I131" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J131" s="2" t="n"/>
       <c r="K131" s="2" t="n"/>
@@ -19171,7 +19171,7 @@
         </is>
       </c>
       <c r="I144" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J144" s="2" t="n"/>
       <c r="K144" s="2" t="n"/>
@@ -19285,7 +19285,7 @@
         </is>
       </c>
       <c r="I148" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J148" s="2" t="n"/>
       <c r="K148" s="2" t="n"/>
@@ -19643,7 +19643,7 @@
         </is>
       </c>
       <c r="I161" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J161" s="2" t="n"/>
       <c r="K161" s="2" t="n"/>
@@ -19757,7 +19757,7 @@
         </is>
       </c>
       <c r="I165" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J165" s="2" t="n"/>
       <c r="K165" s="2" t="n"/>
@@ -20019,7 +20019,7 @@
         </is>
       </c>
       <c r="I175" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J175" s="2" t="n"/>
       <c r="K175" s="2" t="n"/>
@@ -20133,7 +20133,7 @@
         </is>
       </c>
       <c r="I179" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J179" s="2" t="n"/>
       <c r="K179" s="2" t="n"/>
@@ -20247,7 +20247,7 @@
         </is>
       </c>
       <c r="I183" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J183" s="2" t="n"/>
       <c r="K183" s="2" t="n"/>
@@ -20361,7 +20361,7 @@
         </is>
       </c>
       <c r="I187" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J187" s="2" t="n"/>
       <c r="K187" s="2" t="n"/>
@@ -20605,7 +20605,7 @@
         </is>
       </c>
       <c r="I196" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J196" s="2" t="n"/>
       <c r="K196" s="2" t="n"/>
@@ -20719,7 +20719,7 @@
         </is>
       </c>
       <c r="I200" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J200" s="2" t="n"/>
       <c r="K200" s="2" t="n"/>
@@ -21077,7 +21077,7 @@
         </is>
       </c>
       <c r="I213" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J213" s="2" t="n"/>
       <c r="K213" s="2" t="n"/>
@@ -21191,7 +21191,7 @@
         </is>
       </c>
       <c r="I217" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J217" s="2" t="n"/>
       <c r="K217" s="2" t="n"/>
@@ -21549,7 +21549,7 @@
         </is>
       </c>
       <c r="I230" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J230" s="2" t="n"/>
       <c r="K230" s="2" t="n"/>
@@ -21663,7 +21663,7 @@
         </is>
       </c>
       <c r="I234" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J234" s="2" t="n"/>
       <c r="K234" s="2" t="n"/>
@@ -22021,7 +22021,7 @@
         </is>
       </c>
       <c r="I247" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J247" s="2" t="n"/>
       <c r="K247" s="2" t="n"/>
@@ -22135,7 +22135,7 @@
         </is>
       </c>
       <c r="I251" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J251" s="2" t="n"/>
       <c r="K251" s="2" t="n"/>
@@ -22493,7 +22493,7 @@
         </is>
       </c>
       <c r="I264" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J264" s="2" t="n"/>
       <c r="K264" s="2" t="n"/>
@@ -22607,7 +22607,7 @@
         </is>
       </c>
       <c r="I268" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J268" s="2" t="n"/>
       <c r="K268" s="2" t="n"/>
@@ -22965,7 +22965,7 @@
         </is>
       </c>
       <c r="I281" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J281" s="2" t="n"/>
       <c r="K281" s="2" t="n"/>
@@ -23079,7 +23079,7 @@
         </is>
       </c>
       <c r="I285" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J285" s="2" t="n"/>
       <c r="K285" s="2" t="n"/>

</xml_diff>